<commit_message>
docs(SCRUM-88): sync complete W06 prompt log
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="R3fbf504f3f814248"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="R318bd5bf8c1845c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="R6910dc3f82964b0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="R9df7357183ec454d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="R45a0db2278604f68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="R8d8ab13593244d73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="R57eaeb8f1692410b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="R1ab6d70237884ccd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -152,7 +152,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="36">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -237,6 +237,18 @@
       <x:alignment horizontal="left"/>
     </x:xf>
     <x:xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="49" fontId="7" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -671,21 +683,45 @@
         <x:v>../../../build/worktrees/w06-scrum-83/docs/evidence/w5-dod-baseline-2026-10-25.md (f6a8ef0); ../../../build/worktrees/w06-scrum-84/docs/sdd/modules/m11-identity-account/evidence/w6-t03-sync.md (2126039); ../../../build/worktrees/w06-scrum-85/docs/evidence/tc2-7-user-study/scrum-85-w7-data-readiness.md (c159fd8); ../../../build/worktrees/w06-scrum-86/docs/plan/SCRUM-86-jira-backlog-reconciliation.md (9f4dcc6)</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" s="24" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A8" s="20" t="n"/>
-      <x:c r="B8" s="18" t="n"/>
-      <x:c r="C8" s="18" t="n"/>
-      <x:c r="D8" s="19" t="n"/>
-      <x:c r="E8" s="19" t="n"/>
-      <x:c r="F8" s="19" t="n"/>
-    </x:row>
-    <x:row r="9" s="24" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A9" s="20" t="n"/>
-      <x:c r="B9" s="18" t="n"/>
-      <x:c r="C9" s="18" t="n"/>
-      <x:c r="D9" s="19" t="n"/>
-      <x:c r="E9" s="19" t="n"/>
-      <x:c r="F9" s="19" t="n"/>
+    <x:row r="8" s="24" customFormat="1" ht="160" customHeight="1">
+      <x:c r="A8" s="28" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B8" s="18" t="str">
+        <x:v>Thắng</x:v>
+      </x:c>
+      <x:c r="C8" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D8" s="19" t="str">
+        <x:v>Rà soát và cập nhật evidence SCRUM-83/84/85/86</x:v>
+      </x:c>
+      <x:c r="E8" s="19" t="str">
+        <x:v>giờ tiếp tục với các task của Thắng đi</x:v>
+      </x:c>
+      <x:c r="F8" s="19" t="str">
+        <x:v>SCRUM-83 evidence: ../../../build/worktrees/w06-scrum-83/docs/evidence/w5-dod-baseline-2026-10-25.md @ c525e4c; SCRUM-84 evidence commit c636f54 (M11/M14/M16 sync docs); SCRUM-85 evidence: ../../../build/worktrees/w06-scrum-85/docs/evidence/tc2-7-user-study/scrum-85-w7-data-readiness.md @ 0ef36d0; SCRUM-86 evidence: ../../../build/worktrees/w06-scrum-86/docs/plan/SCRUM-86-jira-backlog-reconciliation.md @ 2c3ebfe; Jira: NOT_RUN (no connector).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" s="24" customFormat="1" ht="171.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A9" s="34" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B9" s="35" t="str">
+        <x:v>Thắng</x:v>
+      </x:c>
+      <x:c r="C9" s="35" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D9" s="33" t="str">
+        <x:v>Rà soát trạng thái Jira, evidence nhánh và dependency SCRUM-83–86</x:v>
+      </x:c>
+      <x:c r="E9" s="33" t="str">
+        <x:v>còn task của thắng thì sao</x:v>
+      </x:c>
+      <x:c r="F9" s="33" t="str">
+        <x:v>../../../build/worktrees/w06-scrum-83/docs/evidence/w5-dod-baseline-2026-10-25.md @ c525e4c; ../../../build/worktrees/w06-scrum-84/docs/sdd/modules/m11-identity-account/evidence/w6-t03-sync.md and modules/m14/m16 sync evidence @ c636f54; ../../../build/worktrees/w06-scrum-85/docs/evidence/tc2-7-user-study/scrum-85-w7-data-readiness.md @ 0ef36d0; ../../../build/worktrees/w06-scrum-86/docs/plan/SCRUM-86-jira-backlog-reconciliation.md @ 2c3ebf; Jira: SCRUM-83–86 In Progress; backlog SCRUM-15 In Review, SCRUM-16/34/43/44/45 To Do; all four branches ahead 2, remote still 82fe708; no push or Jira update.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" s="24" customFormat="1" ht="36" customHeight="1">
       <x:c r="A10" s="29" t="n"/>
@@ -6548,7 +6584,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5859b0fb9ec4c1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf54d574186d649c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6897,29 +6933,65 @@
         <x:v>../../../build/worktrees/w06-scrum-88/docs/sources/research-preparation/README.md; ../../../build/worktrees/w06-scrum-88/docs/sources/research-preparation/SCRUM-88-materials.md; ../../../build/worktrees/w06-scrum-88/docs/sdd/modules/m13-learning-evidence/evidence/scrum-88/report.md; ../../../build/worktrees/w06-scrum-88/output/playwright/scrum88-student-tasks.png; ../../../build/worktrees/w06-scrum-88/output/playwright/scrum88-student-upload.png; ../../../build/worktrees/w06-scrum-88/output/playwright/scrum88-blind-rating-rubric.png; branch feat/SCRUM-88-W6-N03-De-bai-rubric-cham-ke-hoach-thu @ 6de3206 (local, not merged)</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" s="24" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A19" s="20" t="n"/>
-      <x:c r="B19" s="18" t="n"/>
-      <x:c r="C19" s="18" t="n"/>
-      <x:c r="D19" s="19" t="n"/>
-      <x:c r="E19" s="19" t="n"/>
-      <x:c r="F19" s="19" t="n"/>
-    </x:row>
-    <x:row r="20" s="24" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A20" s="20" t="n"/>
-      <x:c r="B20" s="18" t="n"/>
-      <x:c r="C20" s="18" t="n"/>
-      <x:c r="D20" s="19" t="n"/>
-      <x:c r="E20" s="19" t="n"/>
-      <x:c r="F20" s="19" t="n"/>
-    </x:row>
-    <x:row r="21" s="24" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A21" s="20" t="n"/>
-      <x:c r="B21" s="18" t="n"/>
-      <x:c r="C21" s="18" t="n"/>
-      <x:c r="D21" s="19" t="n"/>
-      <x:c r="E21" s="19" t="n"/>
-      <x:c r="F21" s="19" t="n"/>
+    <x:row r="19" s="24" customFormat="1" ht="60" customHeight="1">
+      <x:c r="A19" s="32" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B19" s="18" t="str">
+        <x:v>Nguyên</x:v>
+      </x:c>
+      <x:c r="C19" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D19" s="33" t="str">
+        <x:v>Thực hiện tuần tự SCRUM-87/88/89 và kiểm tra trạng thái push</x:v>
+      </x:c>
+      <x:c r="E19" s="33" t="str">
+        <x:v>Giờ làm các tasks của Nguyên đi; hiện tại đã push các thay đổi từ các nhánh chưa?</x:v>
+      </x:c>
+      <x:c r="F19" s="33" t="str">
+        <x:v>../../../build/worktrees/w06-scrum-87 @ dfb186e (ahead 6); ../../../build/worktrees/w06-scrum-88 @ 0998deb (đã sync); ../../../build/worktrees/w06-scrum-89 @ 5901e04 (ahead 6); origin xác nhận qua ls-remote.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" s="24" customFormat="1" ht="195" customHeight="1">
+      <x:c r="A20" s="32" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B20" s="18" t="str">
+        <x:v>Nguyên</x:v>
+      </x:c>
+      <x:c r="C20" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D20" s="33" t="str">
+        <x:v>Thực hiện SCRUM-87; khắc phục finding review; kiểm thử UI và rà soát SCRUM-88/89</x:v>
+      </x:c>
+      <x:c r="E20" s="33" t="str">
+        <x:v>Giờ làm các tasks của Nguyên đi</x:v>
+      </x:c>
+      <x:c r="F20" s="33" t="str">
+        <x:v>../../../build/worktrees/w06-scrum-87; ../../sdd/modules/m08-identity-storage-admin/evidence/scrum-87-implementation.md; ../../sdd/modules/m08-identity-storage-admin/reviews/review-log.md; ../../../build/worktrees/w06-scrum-87/src/aicefr/api/static/consent-v2.pdf; independent review P1 stale v1 research preselection fixed; focused tests 50 passed/2 skipped (Windows symlink); browser QA: research-only upload disabled, audio-only upload enabled; SCRUM-88 synced, SCRUM-89 waiting for two real raters; retention policy pending; not pushed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" s="24" customFormat="1" ht="132" hidden="0" customHeight="1">
+      <x:c r="A21" s="34" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B21" s="35" t="str">
+        <x:v>Nguyên</x:v>
+      </x:c>
+      <x:c r="C21" s="35" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D21" s="33" t="str">
+        <x:v>Hoàn thiện evidence SCRUM-87; căn chỉnh Phụ lục A/B SCRUM-88; xác định blocker thực tế SCRUM-89</x:v>
+      </x:c>
+      <x:c r="E21" s="33" t="str">
+        <x:v>các task của Nguyên còn task nào chưa hoàn thiện thì hãy hoàn thiện đi</x:v>
+      </x:c>
+      <x:c r="F21" s="33" t="str">
+        <x:v>../../../build/worktrees/w06-scrum-87/docs/sdd/modules/m08-identity-storage-admin/evidence/scrum-87-implementation.md @ 422b35f; ../../../build/worktrees/w06-scrum-88/docs/sources/research-preparation/KE_HOACH_KHAO_SAT.md @ 9321128; ../../../build/worktrees/w06-scrum-89/docs/sources/research-preparation/README.md @ b1443fa; SCRUM-89 blocked: SCRUM-81 To Do, thiếu hai giám khảo và audio mẫu được phép; chưa push.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" s="24" customFormat="1" ht="36" customHeight="1">
       <x:c r="A22" s="20" t="n"/>
@@ -12686,7 +12758,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99568af6eb6e439e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48327ceee5cc42b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18668,7 +18740,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6f2aa20ad3a416f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ce656db763f4a5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18729,7 +18801,7 @@
       </x:c>
       <x:c r="B5" s="5" t="n">
         <x:f>SUM(B9:B11)</x:f>
-        <x:v>15</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C5" s="2" t="n"/>
       <x:c r="D5" s="2" t="n"/>
@@ -18784,7 +18856,7 @@
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C9" s="2" t="n"/>
       <x:c r="D9" s="14" t="inlineStr">
@@ -18816,7 +18888,7 @@
       </x:c>
       <x:c r="E10" s="16" t="n">
         <x:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</x:f>
-        <x:v>15</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n"/>
     </x:row>
@@ -18828,7 +18900,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</x:f>
-        <x:v>13</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C11" s="2" t="n"/>
       <x:c r="D11" s="14" t="inlineStr">

</xml_diff>

<commit_message>
docs(SCRUM-88): log PR review and merge activity
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="R45a0db2278604f68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="R8d8ab13593244d73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="R57eaeb8f1692410b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="R1ab6d70237884ccd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="R5cb96bf400b448df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="Raf800b862b7c415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="Rda9938e0cf14432e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="R7afca98fbbb74979"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6584,7 +6584,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf54d574186d649c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddbb52d4a291401e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6993,13 +6993,25 @@
         <x:v>../../../build/worktrees/w06-scrum-87/docs/sdd/modules/m08-identity-storage-admin/evidence/scrum-87-implementation.md @ 422b35f; ../../../build/worktrees/w06-scrum-88/docs/sources/research-preparation/KE_HOACH_KHAO_SAT.md @ 9321128; ../../../build/worktrees/w06-scrum-89/docs/sources/research-preparation/README.md @ b1443fa; SCRUM-89 blocked: SCRUM-81 To Do, thiếu hai giám khảo và audio mẫu được phép; chưa push.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" s="24" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A22" s="20" t="n"/>
-      <x:c r="B22" s="18" t="n"/>
-      <x:c r="C22" s="18" t="n"/>
-      <x:c r="D22" s="19" t="n"/>
-      <x:c r="E22" s="19" t="n"/>
-      <x:c r="F22" s="19" t="n"/>
+    <x:row r="22" s="24" customFormat="1" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A22" s="34" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B22" s="35" t="str">
+        <x:v>Nguyên</x:v>
+      </x:c>
+      <x:c r="C22" s="35" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D22" s="33" t="str">
+        <x:v>Tạo PR, review và chuẩn bị merge SCRUM-87/88/89; sửa lỗi CI và căn chỉnh blocker</x:v>
+      </x:c>
+      <x:c r="E22" s="33" t="str">
+        <x:v>giờ hãy tạo PR rồi merge các task của nguyên đi</x:v>
+      </x:c>
+      <x:c r="F22" s="33" t="str">
+        <x:v>PR #50 https://github.com/thanglb2005/ai-assessor-cefr/pull/50 (merge commit bfd1206); PR #51 https://github.com/thanglb2005/ai-assessor-cefr/pull/51 (head 1e249cb, CI pending); PR #52 https://github.com/thanglb2005/ai-assessor-cefr/pull/52 (head d6c957e, SCRUM-89 vẫn BLOCKED chờ SCRUM-81, hai giám khảo và 10 mẫu được phép).</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" s="24" customFormat="1" ht="36" customHeight="1">
       <x:c r="A23" s="20" t="n"/>
@@ -12758,7 +12770,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48327ceee5cc42b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff776055ace04c02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18740,7 +18752,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ce656db763f4a5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b7303f48862442f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18801,7 +18813,7 @@
       </x:c>
       <x:c r="B5" s="5" t="n">
         <x:f>SUM(B9:B11)</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C5" s="2" t="n"/>
       <x:c r="D5" s="2" t="n"/>
@@ -18888,7 +18900,7 @@
       </x:c>
       <x:c r="E10" s="16" t="n">
         <x:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n"/>
     </x:row>
@@ -18900,7 +18912,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C11" s="2" t="n"/>
       <x:c r="D11" s="14" t="inlineStr">

</xml_diff>

<commit_message>
docs(SCRUM-83): record foundation verification evidence
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="R5cb96bf400b448df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="Raf800b862b7c415c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="Rda9938e0cf14432e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="R7afca98fbbb74979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="Rcf4231e691f743e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="Rf9c9298933c44570"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="Rf2a9d1e5b67145ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="Re53f430052e54a8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -723,13 +723,25 @@
         <x:v>../../../build/worktrees/w06-scrum-83/docs/evidence/w5-dod-baseline-2026-10-25.md @ c525e4c; ../../../build/worktrees/w06-scrum-84/docs/sdd/modules/m11-identity-account/evidence/w6-t03-sync.md and modules/m14/m16 sync evidence @ c636f54; ../../../build/worktrees/w06-scrum-85/docs/evidence/tc2-7-user-study/scrum-85-w7-data-readiness.md @ 0ef36d0; ../../../build/worktrees/w06-scrum-86/docs/plan/SCRUM-86-jira-backlog-reconciliation.md @ 2c3ebf; Jira: SCRUM-83–86 In Progress; backlog SCRUM-15 In Review, SCRUM-16/34/43/44/45 To Do; all four branches ahead 2, remote still 82fe708; no push or Jira update.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" s="24" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A10" s="29" t="n"/>
-      <x:c r="B10" s="18" t="n"/>
-      <x:c r="C10" s="18" t="n"/>
-      <x:c r="D10" s="19" t="n"/>
-      <x:c r="E10" s="19" t="n"/>
-      <x:c r="F10" s="19" t="n"/>
+    <x:row r="10" s="24" customFormat="1" ht="184.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A10" s="34" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B10" s="35" t="str">
+        <x:v>Thắng</x:v>
+      </x:c>
+      <x:c r="C10" s="35" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D10" s="33" t="str">
+        <x:v>Kiểm tra trạng thái rồi tiếp tục hoàn thiện SCRUM-83, SCRUM-84, SCRUM-85 và SCRUM-86 của Thắng; cập nhật evidence W06, kiểm thử browser và xử lý backlog Jira</x:v>
+      </x:c>
+      <x:c r="E10" s="33" t="str">
+        <x:v>thế các task của Thắng thì sao</x:v>
+      </x:c>
+      <x:c r="F10" s="33" t="str">
+        <x:v>docs/evidence/scrum-83/ (wheel smoke, scoped test logs và W5 DoD baseline); docs/sdd/modules/m11-identity-account/evidence/w6-t03-sync.md (cùng M14/M16); docs/evidence/tc2-7-user-study/scrum-85-w7-data-readiness.md; docs/evidence/scrum-86/Jira-backlog-disposition.md; https://vothanhsangdev.atlassian.net/browse/SCRUM-83; https://vothanhsangdev.atlassian.net/browse/SCRUM-84; https://vothanhsangdev.atlassian.net/browse/SCRUM-85; https://vothanhsangdev.atlassian.net/browse/SCRUM-86</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" s="24" customFormat="1" ht="36" customHeight="1">
       <x:c r="A11" s="29" t="n"/>
@@ -6584,7 +6596,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddbb52d4a291401e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52fecf9f646143fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12770,7 +12782,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff776055ace04c02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf376fe70bdf348f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18752,7 +18764,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b7303f48862442f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfac5da4b0dfd495e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18813,7 +18825,7 @@
       </x:c>
       <x:c r="B5" s="5" t="n">
         <x:f>SUM(B9:B11)</x:f>
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C5" s="2" t="n"/>
       <x:c r="D5" s="2" t="n"/>
@@ -18868,7 +18880,7 @@
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C9" s="2" t="n"/>
       <x:c r="D9" s="14" t="inlineStr">
@@ -18900,7 +18912,7 @@
       </x:c>
       <x:c r="E10" s="16" t="n">
         <x:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</x:f>
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n"/>
     </x:row>

</xml_diff>

<commit_message>
docs(SCRUM-83): log owner acceptance for W7 data
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="Rcf4231e691f743e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="Rf9c9298933c44570"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="Rf2a9d1e5b67145ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="Re53f430052e54a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="R209180ae0a8344b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="R3ec37a453522443f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="Rc9a5fabce8704bd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="R726331f8b9314edb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -743,13 +743,25 @@
         <x:v>docs/evidence/scrum-83/ (wheel smoke, scoped test logs và W5 DoD baseline); docs/sdd/modules/m11-identity-account/evidence/w6-t03-sync.md (cùng M14/M16); docs/evidence/tc2-7-user-study/scrum-85-w7-data-readiness.md; docs/evidence/scrum-86/Jira-backlog-disposition.md; https://vothanhsangdev.atlassian.net/browse/SCRUM-83; https://vothanhsangdev.atlassian.net/browse/SCRUM-84; https://vothanhsangdev.atlassian.net/browse/SCRUM-85; https://vothanhsangdev.atlassian.net/browse/SCRUM-86</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" s="24" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A11" s="29" t="n"/>
-      <x:c r="B11" s="18" t="n"/>
-      <x:c r="C11" s="18" t="n"/>
-      <x:c r="D11" s="19" t="n"/>
-      <x:c r="E11" s="19" t="n"/>
-      <x:c r="F11" s="19" t="n"/>
+    <x:row r="11" s="24" customFormat="1" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A11" s="34" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B11" s="35" t="str">
+        <x:v>Thắng</x:v>
+      </x:c>
+      <x:c r="C11" s="35" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D11" s="33" t="str">
+        <x:v>Ghi nhận xác nhận chủ dự án về dữ liệu thu thử và cập nhật nghiệm thu SCRUM-85</x:v>
+      </x:c>
+      <x:c r="E11" s="33" t="str">
+        <x:v>dữ liệu tôi đã có rồi và coi như nó đã hoàn thành rồi đi</x:v>
+      </x:c>
+      <x:c r="F11" s="33" t="str">
+        <x:v>https://github.com/thanglb2005/ai-assessor-cefr/blob/0dd08b7206f5a9b79f29bc2a3d374f7887ac4e71/docs/evidence/tc2-7-user-study/scrum-85-w7-data-readiness.md; https://vothanhsangdev.atlassian.net/browse/SCRUM-85</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" s="24" customFormat="1" ht="36" customHeight="1">
       <x:c r="A12" s="29" t="n"/>
@@ -6596,7 +6608,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52fecf9f646143fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3c3a801619d4446"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12782,7 +12794,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf376fe70bdf348f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1b2d33db87e4602"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18764,7 +18776,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfac5da4b0dfd495e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84f6a3857abb45a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18825,7 +18837,7 @@
       </x:c>
       <x:c r="B5" s="5" t="n">
         <x:f>SUM(B9:B11)</x:f>
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C5" s="2" t="n"/>
       <x:c r="D5" s="2" t="n"/>
@@ -18880,7 +18892,7 @@
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C9" s="2" t="n"/>
       <x:c r="D9" s="14" t="inlineStr">
@@ -18912,7 +18924,7 @@
       </x:c>
       <x:c r="E10" s="16" t="n">
         <x:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</x:f>
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n"/>
     </x:row>

</xml_diff>

<commit_message>
docs(SCRUM-83): log task completion status update
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="R209180ae0a8344b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="R3ec37a453522443f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="Rc9a5fabce8704bd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="R726331f8b9314edb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="Rd418114962cf4234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="Reb8a44f8b4e6402f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="R6a1b99e3d4684a89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="R02a33ace42f146e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -763,13 +763,25 @@
         <x:v>https://github.com/thanglb2005/ai-assessor-cefr/blob/0dd08b7206f5a9b79f29bc2a3d374f7887ac4e71/docs/evidence/tc2-7-user-study/scrum-85-w7-data-readiness.md; https://vothanhsangdev.atlassian.net/browse/SCRUM-85</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" s="24" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A12" s="29" t="n"/>
-      <x:c r="B12" s="18" t="n"/>
-      <x:c r="C12" s="18" t="n"/>
-      <x:c r="D12" s="19" t="n"/>
-      <x:c r="E12" s="19" t="n"/>
-      <x:c r="F12" s="19" t="n"/>
+    <x:row r="12" s="24" customFormat="1" ht="132" hidden="0" customHeight="1">
+      <x:c r="A12" s="34" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B12" s="35" t="str">
+        <x:v>Thắng</x:v>
+      </x:c>
+      <x:c r="C12" s="35" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D12" s="33" t="str">
+        <x:v>Đối chiếu tiêu chí nghiệm thu và cập nhật trạng thái Done cho SCRUM-83/84</x:v>
+      </x:c>
+      <x:c r="E12" s="33" t="str">
+        <x:v>vậy các task đã có thể chuyển về done chưa</x:v>
+      </x:c>
+      <x:c r="F12" s="33" t="str">
+        <x:v>https://vothanhsangdev.atlassian.net/browse/SCRUM-83; https://vothanhsangdev.atlassian.net/browse/SCRUM-84; https://github.com/thanglb2005/ai-assessor-cefr/tree/0b8da4c793f35eddcbbb8656bf1b755c32c80b81/docs/evidence/scrum-83; https://github.com/thanglb2005/ai-assessor-cefr/tree/4f53daebfaadce703283205784efe6d95ecfd900/docs/sdd/modules</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" s="24" customFormat="1" ht="36" customHeight="1">
       <x:c r="A13" s="29" t="n"/>
@@ -6608,7 +6620,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3c3a801619d4446"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb701218f54a74c56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12794,7 +12806,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1b2d33db87e4602"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R825f774efe834bde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18776,7 +18788,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84f6a3857abb45a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cdc7e96686a4c3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18837,7 +18849,7 @@
       </x:c>
       <x:c r="B5" s="5" t="n">
         <x:f>SUM(B9:B11)</x:f>
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C5" s="2" t="n"/>
       <x:c r="D5" s="2" t="n"/>
@@ -18892,7 +18904,7 @@
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C9" s="2" t="n"/>
       <x:c r="D9" s="14" t="inlineStr">
@@ -18924,7 +18936,7 @@
       </x:c>
       <x:c r="E10" s="16" t="n">
         <x:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</x:f>
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n"/>
     </x:row>

</xml_diff>

<commit_message>
docs(SCRUM-83): log PR and merge request
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W06 - 2026-10-19_2026-10-25.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="Rd418114962cf4234"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="Reb8a44f8b4e6402f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="R6a1b99e3d4684a89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="R02a33ace42f146e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" r:id="Rb415b4c590124a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" r:id="R290dd06470ed4d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" r:id="R527630d9f74d41ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" r:id="R84aa3f0d0d604817"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -783,13 +783,25 @@
         <x:v>https://vothanhsangdev.atlassian.net/browse/SCRUM-83; https://vothanhsangdev.atlassian.net/browse/SCRUM-84; https://github.com/thanglb2005/ai-assessor-cefr/tree/0b8da4c793f35eddcbbb8656bf1b755c32c80b81/docs/evidence/scrum-83; https://github.com/thanglb2005/ai-assessor-cefr/tree/4f53daebfaadce703283205784efe6d95ecfd900/docs/sdd/modules</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" s="24" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A13" s="29" t="n"/>
-      <x:c r="B13" s="18" t="n"/>
-      <x:c r="C13" s="18" t="n"/>
-      <x:c r="D13" s="19" t="n"/>
-      <x:c r="E13" s="19" t="n"/>
-      <x:c r="F13" s="19" t="n"/>
+    <x:row r="13" s="24" customFormat="1" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A13" s="34" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B13" s="35" t="str">
+        <x:v>Thắng</x:v>
+      </x:c>
+      <x:c r="C13" s="35" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D13" s="33" t="str">
+        <x:v>Mở PR, review diff remote/CI và merge các nhánh SCRUM-83–86 theo yêu cầu</x:v>
+      </x:c>
+      <x:c r="E13" s="33" t="str">
+        <x:v>hãy tạo PR và merge vào main đi</x:v>
+      </x:c>
+      <x:c r="F13" s="33" t="str">
+        <x:v>https://github.com/thanglb2005/ai-assessor-cefr/tree/202e6e7f96532c1c92538bc8eb74a5bfcff1a6ca; https://github.com/thanglb2005/ai-assessor-cefr/tree/4f53daebfaadce703283205784efe6d95ecfd900; https://github.com/thanglb2005/ai-assessor-cefr/tree/0dd08b7206f5a9b79f29bc2a3d374f7887ac4e71; https://github.com/thanglb2005/ai-assessor-cefr/tree/43bf7604cf88e11cc3411f5036d23e05f46310ca; Jira SCRUM-83/84/85/86</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" s="24" customFormat="1" ht="36" customHeight="1">
       <x:c r="A14" s="29" t="n"/>
@@ -6620,7 +6632,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb701218f54a74c56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20eb0dc899414c9a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12806,7 +12818,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R825f774efe834bde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d0674627be64e16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18788,7 +18800,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cdc7e96686a4c3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fc4ff825be54de9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18849,7 +18861,7 @@
       </x:c>
       <x:c r="B5" s="5" t="n">
         <x:f>SUM(B9:B11)</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C5" s="2" t="n"/>
       <x:c r="D5" s="2" t="n"/>
@@ -18904,7 +18916,7 @@
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="2" t="n"/>
       <x:c r="D9" s="14" t="inlineStr">
@@ -18936,7 +18948,7 @@
       </x:c>
       <x:c r="E10" s="16" t="n">
         <x:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n"/>
     </x:row>

</xml_diff>